<commit_message>
Stage 8 review fixes: E-012
</commit_message>
<xml_diff>
--- a/output/archive/WestravelleData/Methods/XE2/WA-2026-275/Results/Interim/XE2_FIRST_PULL_REVIEW_DRAFT_Rev01.xlsx
+++ b/output/archive/WestravelleData/Methods/XE2/WA-2026-275/Results/Interim/XE2_FIRST_PULL_REVIEW_DRAFT_Rev01.xlsx
@@ -19,13 +19,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -80,16 +84,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -173,14 +178,14 @@
     <author>Saira Mahmood</author>
   </authors>
   <commentList>
-    <comment ref="E5" authorId="0" shapeId="0">
+    <comment ref="B6" authorId="0" shapeId="0">
       <text>
-        <t>Shoulder is the same width in the acid and peroxide samples. Do not integrate it into the main peak until the rule is agreed.</t>
+        <t>Agree the shoulder-peak integration rule before validation sign-off.</t>
       </text>
     </comment>
-    <comment ref="A9" authorId="1" shapeId="0">
+    <comment ref="B7" authorId="1" shapeId="0">
       <text>
-        <t>Hydrolysis control row is empty. Leon to confirm whether the control was run in this sequence or the next.</t>
+        <t>Keep the specificity conclusion pending until the integration review is complete.</t>
       </text>
     </comment>
   </commentList>
@@ -476,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -487,190 +492,197 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>WA/2026/275 XE2 assay validation: INTERIM DRAFT</t>
+          <t>Westravelle Analytical Ltd, a Tarnovell company</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>WA/2026/275 XE2 assay validation: INTERIM DRAFT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>Status: interim. Forced degradation complete; integration rules and validation sign-off pending.</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>WA/2026/275</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>LIMS</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>WST-26-008543</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Xelvessune Pharma</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Lead</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Alice Penrose</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Method validation</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Saira Mahmood</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Sequence owner</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Leon Wu</t>
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Quote accepted</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>11/08/2026</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Protocol start</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>08/09/2026</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Interim data review</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>29/09/2026</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Completion</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>To be confirmed</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Result (interim)</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Overall outcome so far</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Specificity established for the stressed samples at the peaks already integrated; shoulder peak under review</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Forced-degradation work complete; shoulder-peak integration rules and validation sign-off pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Prepared by</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Saira Mahmood</t>
         </is>
       </c>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="C21" s="3" t="n"/>
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>Interim draft 29/09/2026</t>
         </is>
@@ -691,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -704,234 +716,113 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Forced degradation: specificity sequence (interim)</t>
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Forced-degradation review tracker (interim)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Stress conditions as per protocol. Peak purity assessed on the main peak in every stressed sample. Blank cells are results not yet reviewed.</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Forced-degradation work is complete. Stress settings, chromatograms and peak assessments remain in the source sequence records; blank cells below are pending review or sign-off entries.</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Stress condition</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Protocol setting</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Exposure</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Main peak purity</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Shoulder peak</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Integration reviewed</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Comment</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Review item</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Reviewer</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Sign-off</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Acid</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>0.1 M HCl, 60 °C</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Forced-degradation work</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Integration rule being set</t>
-        </is>
-      </c>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>0.1 M NaOH, 60 °C</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Not seen</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>No action</t>
-        </is>
-      </c>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Shoulder-peak integration rules</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Being finalised</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Saira Mahmood</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Peroxide</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>3% H2O2, room temperature</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Same shoulder as acid sample</t>
-        </is>
-      </c>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Specificity conclusion</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Heat (solid)</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>80 °C, 7 days</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Validation sign-off</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Light</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>ICH Q1B exposure</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Hydrolysis control</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Water, 60 °C</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Report issue</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -958,14 +849,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>HPLC method qualification: interim parameters</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Parameters run to date. Specificity and robustness not yet signed off; see forced degradation sheet.</t>
         </is>
@@ -973,94 +864,94 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Acceptance</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Linearity (r²)</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>0.9995000000000001</v>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>≥0.999</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Range (% nominal)</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>50-150</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>80-120 minimum</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Accuracy 80% (% recovery)</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="3" t="n">
         <v>99.8</v>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>98.0-102.0</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Accuracy 100% (% recovery)</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="3" t="n">
         <v>100.4</v>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>98.0-102.0</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Accuracy 120% (% recovery)</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="3" t="n">
         <v>99.90000000000001</v>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>98.0-102.0</t>
         </is>
@@ -1068,7 +959,7 @@
     </row>
     <row r="10"/>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>INTERIM: 5 of 8 planned rows reported; remaining in progress</t>
         </is>

</xml_diff>